<commit_message>
chore(eca): 2026-07 월간 업데이트
</commit_message>
<xml_diff>
--- a/docs/archive/2026-07/2026-07_ECA_기록.xlsx
+++ b/docs/archive/2026-07/2026-07_ECA_기록.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="172">
   <si>
     <t>id</t>
   </si>
@@ -58,6 +58,78 @@
     <t>게시상태</t>
   </si>
   <si>
+    <t>children-product-safety-drawing-contest-2026</t>
+  </si>
+  <si>
+    <t>2026 어린이 제품안전 그림공모전</t>
+  </si>
+  <si>
+    <t>환경·예술·공익</t>
+  </si>
+  <si>
+    <t>예술·디자인</t>
+  </si>
+  <si>
+    <t>유치부(2020~2022년생), 초등부(2014~2019년생)</t>
+  </si>
+  <si>
+    <t>산업통상부 국가기술표준원, 한국제품안전관리원</t>
+  </si>
+  <si>
+    <t>2026-07-24</t>
+  </si>
+  <si>
+    <t>무료</t>
+  </si>
+  <si>
+    <t>낮음</t>
+  </si>
+  <si>
+    <t>★★★</t>
+  </si>
+  <si>
+    <t>공모전, 무료, 개인</t>
+  </si>
+  <si>
+    <t>https://kips.kr/kips.do</t>
+  </si>
+  <si>
+    <t>제품안전을 주제로 한 그림(8절 도화지 손그림, 포스터·만화 등 자유형식)을 겨루는 정부 주최 어린이 그림공모전.</t>
+  </si>
+  <si>
+    <t>게시</t>
+  </si>
+  <si>
+    <t>global-citizen-photo-essay-2026</t>
+  </si>
+  <si>
+    <t>지금, 세계시민 ON 포토에세이 공모전</t>
+  </si>
+  <si>
+    <t>국제·리더십·사회참여</t>
+  </si>
+  <si>
+    <t>사회·정책, 국제·외교, 예술·디자인</t>
+  </si>
+  <si>
+    <t>국적과 관계없이 국내에 거주하는 초·중·고생 또는 동일 연령대 청소년</t>
+  </si>
+  <si>
+    <t>외교부, 유네스코 아시아태평양 국제이해교육원(유네스코 아태교육원)</t>
+  </si>
+  <si>
+    <t>2026-07-26</t>
+  </si>
+  <si>
+    <t>공모전, 에세이·논문, 무료, 전국규모, 개인</t>
+  </si>
+  <si>
+    <t>https://www.unescoapceiu.org/</t>
+  </si>
+  <si>
+    <t>세계시민 가치를 사진과 에세이로 표현하는 외교부·유네스코 아태교육원 공동 주최 청소년 공모전.</t>
+  </si>
+  <si>
     <t>the-concord-review-2026</t>
   </si>
   <si>
@@ -67,7 +139,7 @@
     <t>글쓰기·논문·인문사회</t>
   </si>
   <si>
-    <t>인문, 역사</t>
+    <t>인문·철학, 사회·정책</t>
   </si>
   <si>
     <t>중등교육(고교) 졸업 이전에 논문을 완성한 학생</t>
@@ -88,16 +160,13 @@
     <t>★★★★</t>
   </si>
   <si>
-    <t>에세이·논문, 연구, 인문·철학, 개인, 국제대회</t>
+    <t>에세이·논문, 연구, 국제대회, 개인</t>
   </si>
   <si>
     <t>https://tcr.org/submit</t>
   </si>
   <si>
-    <t>고교생 역사 연구논문을 심사·게재하는 국제 학술지. 게재율 약 5%.</t>
-  </si>
-  <si>
-    <t>게시</t>
+    <t>고교생 역사 연구논문을 심사·게재하는 국제 학술지.</t>
   </si>
   <si>
     <t>environment-love-contest-2026</t>
@@ -106,124 +175,328 @@
     <t>2026 대한민국 환경사랑공모전</t>
   </si>
   <si>
-    <t>환경·예술·공익</t>
-  </si>
-  <si>
-    <t>환경, 예술</t>
+    <t>환경, 예술·디자인</t>
   </si>
   <si>
     <t>신청자격 제한 없음(대한민국 국민 누구나). 일러스트레이션 부문은 학생부(초등부/중·고등부) 별도 운영.</t>
   </si>
   <si>
-    <t>한국환경공단 (공식 페이지 연관 기관)</t>
+    <t>한국환경공단</t>
   </si>
   <si>
     <t>2026-08-03</t>
   </si>
   <si>
-    <t>무료</t>
+    <t>공모전, 무료, 전국규모, 개인</t>
+  </si>
+  <si>
+    <t>https://xn--289a5d925ap8c64jnzlpiz.kr/</t>
+  </si>
+  <si>
+    <t>사진·에코디자인·일러스트레이션 부문으로 환경 인식을 겨루는 전국 규모 환경 공모전.</t>
+  </si>
+  <si>
+    <t>hir-academic-writing-contest-2026</t>
+  </si>
+  <si>
+    <t>Harvard International Review Academic Writing Contest 2026</t>
+  </si>
+  <si>
+    <t>인문·철학, 사회·정책, 국제·외교</t>
+  </si>
+  <si>
+    <t>7~12학년 학생(미국 외 국가 학생 포함)</t>
+  </si>
+  <si>
+    <t>Harvard International Review (HIR)</t>
+  </si>
+  <si>
+    <t>2026-08-24</t>
+  </si>
+  <si>
+    <t>에세이·논문, 공모전, 국제대회, 개인</t>
+  </si>
+  <si>
+    <t>https://hir.harvard.edu/contest/</t>
+  </si>
+  <si>
+    <t>국제관계·외교 주제의 단편 학술 아티클을 겨루는 하버드국제리뷰 주최 글쓰기 대회.</t>
+  </si>
+  <si>
+    <t>fss-financial-contest-2026</t>
+  </si>
+  <si>
+    <t>제21회 금융공모전 (청소년 금융창작물 부문 등)</t>
+  </si>
+  <si>
+    <t>경제·금융, 미디어·영상</t>
+  </si>
+  <si>
+    <t>초·중·고등학교 재학생과 동일 연령대 청소년 (청소년 부문). 대학생·성인·기관 부문도 별도 운영.</t>
+  </si>
+  <si>
+    <t>금융감독원</t>
+  </si>
+  <si>
+    <t>2026-09-02</t>
+  </si>
+  <si>
+    <t>https://www.fss.or.kr/edu</t>
+  </si>
+  <si>
+    <t>금융에 대한 관심과 이해를 높이기 위해 글짓기·UCC·포스터·만화 등으로 참여하는 금융감독원 주최 전 국민 대상 공모전(청소년 부문 별도 운영).</t>
+  </si>
+  <si>
+    <t>breakthrough-junior-challenge-2026</t>
+  </si>
+  <si>
+    <t>Breakthrough Junior Challenge 2026</t>
+  </si>
+  <si>
+    <t>과학·공학·수학생명·AI</t>
+  </si>
+  <si>
+    <t>과학, 물리·화학, 생명·의학, 수학, 미디어·영상</t>
+  </si>
+  <si>
+    <t>만 13~18세 학생(2026-05-11 기준 13세 이상, 2026-10-01 기준 만 19세 미만). 개인 참가만 가능.</t>
+  </si>
+  <si>
+    <t>Breakthrough Prize Foundation</t>
+  </si>
+  <si>
+    <t>2026-09-15</t>
+  </si>
+  <si>
+    <t>★★★★★</t>
+  </si>
+  <si>
+    <t>공모전, 국제대회, 개인, 무료, 미디어·영상</t>
+  </si>
+  <si>
+    <t>https://breakthroughjuniorchallenge.org/</t>
+  </si>
+  <si>
+    <t>생명과학·물리·수학 개념을 짧은 영상으로 설명하는 국제 대회(개인전).</t>
+  </si>
+  <si>
+    <t>amc-2026</t>
+  </si>
+  <si>
+    <t>AMC (American Mathematics Competitions) 2026</t>
+  </si>
+  <si>
+    <t>수학</t>
+  </si>
+  <si>
+    <t>중·고등학생 (AMC 8: 8학년 이하 / AMC 10: 10학년 이하 / AMC 12: 12학년 이하)</t>
+  </si>
+  <si>
+    <t>MAA (Mathematical Association of America)</t>
+  </si>
+  <si>
+    <t>2026-09-30</t>
+  </si>
+  <si>
+    <t>올림피아드, 국제대회, 개인</t>
+  </si>
+  <si>
+    <t>https://maa.org/amcreg/</t>
+  </si>
+  <si>
+    <t>MAA가 주최하는 국제 수학경시대회. AMC 8/10/12로 나뉘며 상위자는 AIME·USA(J)MO 선발 경로로 이어진다.</t>
+  </si>
+  <si>
+    <t>iearn</t>
+  </si>
+  <si>
+    <t>iEARN (International Education and Resource Network) 글로벌 협업 프로젝트</t>
+  </si>
+  <si>
+    <t>사회·정책, 국제·외교, 문화</t>
+  </si>
+  <si>
+    <t>전 세계 학생·교사(초·중·고 및 청소년 기관)</t>
+  </si>
+  <si>
+    <t>iEARN (International Education and Resource Network, 1988년 설립 비영리 국제교육네트워크)</t>
+  </si>
+  <si>
+    <t>상시</t>
+  </si>
+  <si>
+    <t>온라인, 상시모집, 팀, 국제대회</t>
+  </si>
+  <si>
+    <t>https://iearn.org/</t>
+  </si>
+  <si>
+    <t>140개국 학교가 참여하는 국제 협업·가상교류 프로젝트 네트워크. 한국(iEARN-South Korea)도 참여국.</t>
+  </si>
+  <si>
+    <t>nasa-citizen-science</t>
+  </si>
+  <si>
+    <t>NASA Citizen Science (시민과학 프로젝트)</t>
+  </si>
+  <si>
+    <t>과학, 공학</t>
+  </si>
+  <si>
+    <t>누구나(시민권 불필요). 청소년 포함 전 세계 참여자.</t>
+  </si>
+  <si>
+    <t>NASA (미국 항공우주국)</t>
   </si>
   <si>
     <t>보통</t>
   </si>
   <si>
-    <t>공모전, 환경, 예술·디자인, 무료, 전국규모</t>
-  </si>
-  <si>
-    <t>https://xn--289a5d925ap8c64jnzlpiz.kr/</t>
-  </si>
-  <si>
-    <t>사진·에코디자인·일러스트레이션 부문으로 환경 인식을 겨루는 전국 규모 환경 공모전.</t>
-  </si>
-  <si>
-    <t>hir-academic-writing-contest-2026</t>
-  </si>
-  <si>
-    <t>Harvard International Review Academic Writing Contest 2026</t>
-  </si>
-  <si>
-    <t>인문, 사회</t>
-  </si>
-  <si>
-    <t>7~12학년 학생(미국 외 국가 학생 포함)</t>
-  </si>
-  <si>
-    <t>Harvard International Review (HIR)</t>
-  </si>
-  <si>
-    <t>2026-08-24</t>
-  </si>
-  <si>
-    <t>에세이·논문, 국제·외교, 사회·정책, 개인, 국제대회</t>
-  </si>
-  <si>
-    <t>https://hir.harvard.edu/contest/</t>
-  </si>
-  <si>
-    <t>국제관계·외교 주제의 단편 학술 아티클을 겨루는 하버드국제리뷰 주최 글쓰기 대회.</t>
-  </si>
-  <si>
-    <t>breakthrough-junior-challenge-2026</t>
-  </si>
-  <si>
-    <t>Breakthrough Junior Challenge 2026</t>
-  </si>
-  <si>
-    <t>과학·공학·수학생명·AI</t>
-  </si>
-  <si>
-    <t>과학, 수학</t>
-  </si>
-  <si>
-    <t>만 13~18세 학생(2026-05-11 기준 13세 이상, 2026-10-01 기준 만 19세 미만). 개인 참가만 가능.</t>
-  </si>
-  <si>
-    <t>Breakthrough Prize Foundation</t>
-  </si>
-  <si>
-    <t>2026-09-15</t>
-  </si>
-  <si>
-    <t>★★★★★</t>
-  </si>
-  <si>
-    <t>공모전, 과학, 생명·의학, 미디어·영상, 무료, 개인, 국제대회</t>
-  </si>
-  <si>
-    <t>https://breakthroughjuniorchallenge.org/</t>
-  </si>
-  <si>
-    <t>생명과학·물리·수학 개념을 2분 이내 영상으로 설명하는 국제 대회(개인전).</t>
-  </si>
-  <si>
-    <t>amc-2026</t>
-  </si>
-  <si>
-    <t>AMC (American Mathematics Competitions) 2026</t>
-  </si>
-  <si>
-    <t>수학</t>
-  </si>
-  <si>
-    <t>중·고등학생 (AMC 8: 8학년 이하 / AMC 10: 10학년 이하 / AMC 12: 12학년 이하)</t>
-  </si>
-  <si>
-    <t>MAA (Mathematical Association of America)</t>
-  </si>
-  <si>
-    <t>2026-10-28</t>
-  </si>
-  <si>
-    <t>★★★</t>
-  </si>
-  <si>
-    <t>올림피아드, 수학, 국제대회, 개인</t>
-  </si>
-  <si>
-    <t>https://maa.org/amcreg/</t>
-  </si>
-  <si>
-    <t>MAA가 주최하는 국제 수학경시대회. AMC 8/10/12로 나뉘며 상위자는 AIME·USA(J)MO 선발 경로로 이어진다.</t>
+    <t>연구, 온라인, 무료, 국제대회, 개인</t>
+  </si>
+  <si>
+    <t>https://science.nasa.gov/citizen-science/</t>
+  </si>
+  <si>
+    <t>NASA 연구진과 함께 천문·지구과학 등 실제 과학 프로젝트에 자원 참여하는 시민과학 프로그램.</t>
+  </si>
+  <si>
+    <t>roots-and-shoots</t>
+  </si>
+  <si>
+    <t>Roots &amp; Shoots (제인 구달 청소년 봉사·환경 프로그램)</t>
+  </si>
+  <si>
+    <t>스포츠·문화·봉사</t>
+  </si>
+  <si>
+    <t>환경</t>
+  </si>
+  <si>
+    <t>전 세계 청소년(young people). 초·중·고 포함.</t>
+  </si>
+  <si>
+    <t>Jane Goodall Institute (제인 구달 박사 설립)</t>
+  </si>
+  <si>
+    <t>★★</t>
+  </si>
+  <si>
+    <t>봉사, 환경, 무료, 팀, 상시모집</t>
+  </si>
+  <si>
+    <t>https://rootsandshoots.org/</t>
+  </si>
+  <si>
+    <t>제인구달연구소가 운영하는 청소년 주도 지역사회 봉사·환경·동물복지 프로젝트 프로그램(글로벌 챕터).</t>
+  </si>
+  <si>
+    <t>globe-program</t>
+  </si>
+  <si>
+    <t>The GLOBE Program (국제 환경 관측·교육 프로그램)</t>
+  </si>
+  <si>
+    <t>환경, 과학</t>
+  </si>
+  <si>
+    <t>초등~고등 학생 및 교사(환경 데이터 수집 참여)</t>
+  </si>
+  <si>
+    <t>NASA 후원, NSF·NOAA·미 국무부 지원</t>
+  </si>
+  <si>
+    <t>연구, 캠프·체험, 상시모집, 무료, 국제대회</t>
+  </si>
+  <si>
+    <t>https://www.globe.gov/</t>
+  </si>
+  <si>
+    <t>전 세계 학생이 표준 프로토콜로 환경 데이터를 관측·공유하는 NASA 후원 국제 환경 과학·교육 프로그램. 한국(Republic of Korea)도 참여국.</t>
+  </si>
+  <si>
+    <t>wharton-investment-competition-2027</t>
+  </si>
+  <si>
+    <t>Wharton Global High School Investment Competition (2026-2027)</t>
+  </si>
+  <si>
+    <t>경제·금융</t>
+  </si>
+  <si>
+    <t>고등학생(9~12학년), 교사 지도 하 4~6인 팀</t>
+  </si>
+  <si>
+    <t>Wharton Global Youth Program, University of Pennsylvania</t>
+  </si>
+  <si>
+    <t>공모전, 국제대회, 팀</t>
+  </si>
+  <si>
+    <t>https://globalyouth.wharton.upenn.edu/competitions/investment-competition/</t>
+  </si>
+  <si>
+    <t>모의 주식 포트폴리오를 운용하고 투자전략 보고서를 겨루는 와튼 주최 글로벌 고교 투자대회(팀전).</t>
+  </si>
+  <si>
+    <t>world-scholars-cup-2026</t>
+  </si>
+  <si>
+    <t>World Scholar's Cup 2026 (Korea Round, Seoul Global Round)</t>
+  </si>
+  <si>
+    <t>초·중·고 학생(팀 참가), 국가/지역별 라운드 참가</t>
+  </si>
+  <si>
+    <t>World Scholar's Cup</t>
+  </si>
+  <si>
+    <t>토론·스피치, 공모전, 국제대회, 팀</t>
+  </si>
+  <si>
+    <t>https://www.scholarscup.org/</t>
+  </si>
+  <si>
+    <t>토론·에세이·퀴즈·협동 프레젠테이션 등을 겨루는 국제 학술 대회. 한국(서울) 라운드가 매년 개최된다.</t>
+  </si>
+  <si>
+    <t>zooniverse</t>
+  </si>
+  <si>
+    <t>Zooniverse (온라인 시민과학 연구 참여)</t>
+  </si>
+  <si>
+    <t>과학, 생명·의학</t>
+  </si>
+  <si>
+    <t>누구나(전문 배경·훈련 불필요). 16세 미만은 보호자 동의 하 계정 생성 가능.</t>
+  </si>
+  <si>
+    <t>The Zooniverse (Adler Planetarium, University of Minnesota, University of Oxford 파트너)</t>
+  </si>
+  <si>
+    <t>https://www.zooniverse.org/</t>
+  </si>
+  <si>
+    <t>천문·생태·기후 등 실제 연구 데이터를 자원자가 분류·분석하는 세계 최대 시민과학 플랫폼.</t>
+  </si>
+  <si>
+    <t>구분</t>
+  </si>
+  <si>
+    <t>사유/마감일</t>
+  </si>
+  <si>
+    <t>게시 제외</t>
+  </si>
+  <si>
+    <t>seoul-environmental-education-content-contest-2026</t>
+  </si>
+  <si>
+    <t>2026년 제3회 서울특별시 환경교육 콘텐츠 공모전</t>
+  </si>
+  <si>
+    <t>제외(링크오류: UNABLE_TO_VERIFY_LEAF_SIGNATURE)</t>
   </si>
   <si>
     <t>1365-volunteer-portal</t>
@@ -232,184 +505,13 @@
     <t>1365 자원봉사포털 청소년 자원봉사</t>
   </si>
   <si>
-    <t>스포츠·문화·봉사</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>청소년(초·중·고 포함) 및 일반 국민</t>
-  </si>
-  <si>
-    <t>행정안전부 (재단법인 한국중앙자원봉사센터 운영)</t>
-  </si>
-  <si>
-    <t>상시</t>
-  </si>
-  <si>
-    <t>낮음</t>
-  </si>
-  <si>
-    <t>봉사, 무료, 상시모집, 전국규모</t>
-  </si>
-  <si>
-    <t>https://www.1365.go.kr/vols/main.do</t>
-  </si>
-  <si>
-    <t>전국 자원봉사 정보를 통합 제공하는 정부 포털. 검색·신청·실적 확인·확인서 발급을 원스톱 제공하며 NEIS 연계로 학생부 반영.</t>
-  </si>
-  <si>
-    <t>iearn</t>
-  </si>
-  <si>
-    <t>iEARN (International Education and Resource Network) 글로벌 협업 프로젝트</t>
-  </si>
-  <si>
-    <t>국제·리더십·사회참여</t>
-  </si>
-  <si>
-    <t>국제, 사회</t>
-  </si>
-  <si>
-    <t>전 세계 학생·교사(초·중·고 및 청소년 기관)</t>
-  </si>
-  <si>
-    <t>iEARN (International Education and Resource Network, 1988년 설립 비영리 국제교육네트워크)</t>
-  </si>
-  <si>
-    <t>★★</t>
-  </si>
-  <si>
-    <t>온라인, 국제·외교, 사회·정책, 팀, 상시모집</t>
-  </si>
-  <si>
-    <t>https://iearn.org/</t>
-  </si>
-  <si>
-    <t>140개국 학교가 참여하는 국제 협업·가상교류 프로젝트 네트워크. 학생이 사회문제 해결형 글로벌 프로젝트를 기획·참여.</t>
-  </si>
-  <si>
-    <t>nasa-citizen-science</t>
-  </si>
-  <si>
-    <t>NASA Citizen Science (시민과학 프로젝트)</t>
-  </si>
-  <si>
-    <t>과학</t>
-  </si>
-  <si>
-    <t>누구나(시민권 불필요). 청소년 포함 전 세계 참여자.</t>
-  </si>
-  <si>
-    <t>NASA (미국 항공우주국)</t>
-  </si>
-  <si>
-    <t>연구, 온라인, 과학, 무료, 상시모집</t>
-  </si>
-  <si>
-    <t>https://science.nasa.gov/citizen-science/</t>
-  </si>
-  <si>
-    <t>NASA 연구진과 함께 천문·지구과학 등 실제 과학 프로젝트에 자원 참여하는 시민과학 프로그램(46개 프로젝트 운영).</t>
-  </si>
-  <si>
-    <t>roots-and-shoots</t>
-  </si>
-  <si>
-    <t>Roots &amp; Shoots (제인 구달 청소년 봉사·환경 프로그램)</t>
-  </si>
-  <si>
-    <t>환경</t>
-  </si>
-  <si>
-    <t>전 세계 청소년(young people). 초·중·고 포함.</t>
-  </si>
-  <si>
-    <t>Jane Goodall Institute (제인 구달 박사 설립)</t>
-  </si>
-  <si>
-    <t>봉사, 환경, 무료, 팀, 상시모집</t>
-  </si>
-  <si>
-    <t>https://rootsandshoots.org/</t>
-  </si>
-  <si>
-    <t>제인구달연구소가 운영하는 청소년 주도 지역사회 봉사·환경·동물복지 프로젝트 프로그램(글로벌 챕터).</t>
-  </si>
-  <si>
-    <t>globe-program</t>
-  </si>
-  <si>
-    <t>The GLOBE Program (국제 환경 관측·교육 프로그램)</t>
-  </si>
-  <si>
-    <t>환경, 과학</t>
-  </si>
-  <si>
-    <t>초등~고등 학생 및 상위 교육단계(환경 데이터 수집 참여)</t>
-  </si>
-  <si>
-    <t>NASA 후원, NSF·NOAA·미 국무부 지원</t>
-  </si>
-  <si>
-    <t>연구, 온라인, 환경, 과학, 무료, 상시모집</t>
-  </si>
-  <si>
-    <t>https://www.globe.gov/</t>
-  </si>
-  <si>
-    <t>전 세계 학생이 표준 프로토콜로 환경 데이터를 관측·공유하는 NASA 후원 국제 환경 과학·교육 프로그램.</t>
-  </si>
-  <si>
-    <t>wharton-investment-competition-2027</t>
-  </si>
-  <si>
-    <t>Wharton Global High School Investment Competition (2026-2027)</t>
-  </si>
-  <si>
-    <t>경제, 금융</t>
-  </si>
-  <si>
-    <t>고등학생(9~12학년), 교사 지도 하 4~6인 팀</t>
-  </si>
-  <si>
-    <t>Wharton Global Youth Program, University of Pennsylvania</t>
-  </si>
-  <si>
-    <t>공모전, 경제·금융, 팀, 국제대회</t>
-  </si>
-  <si>
-    <t>https://globalyouth.wharton.upenn.edu/competitions/investment-competition/</t>
-  </si>
-  <si>
-    <t>모의 주식 포트폴리오를 운용하고 투자전략 보고서를 겨루는 와튼 주최 글로벌 고교 투자대회(팀전).</t>
-  </si>
-  <si>
-    <t>zooniverse</t>
-  </si>
-  <si>
-    <t>Zooniverse (온라인 시민과학 연구 참여)</t>
-  </si>
-  <si>
-    <t>누구나(전문 배경·훈련 불필요). 초·중·고 포함 전 연령.</t>
-  </si>
-  <si>
-    <t>The Zooniverse (Adler Planetarium, University of Minnesota, University of Oxford 파트너)</t>
-  </si>
-  <si>
-    <t>연구, 온라인, 과학, 무료, 개인, 상시모집</t>
-  </si>
-  <si>
-    <t>https://www.zooniverse.org/</t>
-  </si>
-  <si>
-    <t>천문·생태·기후 등 실제 연구 데이터를 자원자가 분류·분석하는 세계 최대 시민과학 플랫폼.</t>
-  </si>
-  <si>
-    <t>구분</t>
-  </si>
-  <si>
-    <t>사유/마감일</t>
+    <t>제외(링크오류: UND_ERR_CONNECT_TIMEOUT)</t>
+  </si>
+  <si>
+    <t>duke-of-edinburgh-award-korea</t>
+  </si>
+  <si>
+    <t>국제청소년성취포상제 (The Duke of Edinburgh's International Award, Korea)</t>
   </si>
   <si>
     <t>게시 건수</t>
@@ -816,18 +918,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="37" customWidth="1"/>
+    <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
     <col min="5" max="6" width="60" customWidth="1"/>
     <col min="7" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="13" width="60" customWidth="1"/>
+    <col min="11" max="11" width="44" customWidth="1"/>
+    <col min="12" max="13" width="60" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -942,22 +1045,22 @@
         <v>34</v>
       </c>
       <c r="H3" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="J3" t="s">
         <v>23</v>
       </c>
       <c r="K3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" t="s">
         <v>37</v>
-      </c>
-      <c r="L3" t="s">
-        <v>38</v>
-      </c>
-      <c r="M3" t="s">
-        <v>39</v>
       </c>
       <c r="N3" t="s">
         <v>27</v>
@@ -965,43 +1068,43 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
         <v>40</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>41</v>
       </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>42</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>43</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>44</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>45</v>
       </c>
-      <c r="H4" t="s">
-        <v>21</v>
-      </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="J4" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="K4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="L4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="M4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="N4" t="s">
         <v>27</v>
@@ -1009,34 +1112,34 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="I5" t="s">
         <v>22</v>
       </c>
       <c r="J5" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="K5" t="s">
         <v>57</v>
@@ -1059,7 +1162,7 @@
         <v>61</v>
       </c>
       <c r="C6" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
         <v>62</v>
@@ -1074,22 +1177,22 @@
         <v>65</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I6" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="J6" t="s">
+        <v>47</v>
+      </c>
+      <c r="K6" t="s">
         <v>66</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>67</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>68</v>
-      </c>
-      <c r="M6" t="s">
-        <v>69</v>
       </c>
       <c r="N6" t="s">
         <v>27</v>
@@ -1097,43 +1200,43 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" t="s">
         <v>70</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
         <v>71</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>72</v>
       </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>74</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" t="s">
         <v>75</v>
       </c>
-      <c r="G7" t="s">
+      <c r="M7" t="s">
         <v>76</v>
-      </c>
-      <c r="H7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" t="s">
-        <v>77</v>
-      </c>
-      <c r="J7" t="s">
-        <v>66</v>
-      </c>
-      <c r="K7" t="s">
-        <v>78</v>
-      </c>
-      <c r="L7" t="s">
-        <v>79</v>
-      </c>
-      <c r="M7" t="s">
-        <v>80</v>
       </c>
       <c r="N7" t="s">
         <v>27</v>
@@ -1141,43 +1244,43 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" t="s">
         <v>81</v>
       </c>
-      <c r="B8" t="s">
+      <c r="F8" t="s">
         <v>82</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
         <v>83</v>
-      </c>
-      <c r="D8" t="s">
-        <v>84</v>
-      </c>
-      <c r="E8" t="s">
-        <v>85</v>
-      </c>
-      <c r="F8" t="s">
-        <v>86</v>
-      </c>
-      <c r="G8" t="s">
-        <v>76</v>
       </c>
       <c r="H8" t="s">
         <v>21</v>
       </c>
       <c r="I8" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="J8" t="s">
+        <v>84</v>
+      </c>
+      <c r="K8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L8" t="s">
+        <v>86</v>
+      </c>
+      <c r="M8" t="s">
         <v>87</v>
-      </c>
-      <c r="K8" t="s">
-        <v>88</v>
-      </c>
-      <c r="L8" t="s">
-        <v>89</v>
-      </c>
-      <c r="M8" t="s">
-        <v>90</v>
       </c>
       <c r="N8" t="s">
         <v>27</v>
@@ -1185,43 +1288,43 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" t="s">
         <v>91</v>
       </c>
-      <c r="B9" t="s">
+      <c r="F9" t="s">
         <v>92</v>
       </c>
-      <c r="C9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="G9" t="s">
         <v>93</v>
       </c>
-      <c r="E9" t="s">
+      <c r="H9" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" t="s">
         <v>94</v>
       </c>
-      <c r="F9" t="s">
+      <c r="L9" t="s">
         <v>95</v>
       </c>
-      <c r="G9" t="s">
-        <v>76</v>
-      </c>
-      <c r="H9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I9" t="s">
-        <v>36</v>
-      </c>
-      <c r="J9" t="s">
-        <v>23</v>
-      </c>
-      <c r="K9" t="s">
+      <c r="M9" t="s">
         <v>96</v>
-      </c>
-      <c r="L9" t="s">
-        <v>97</v>
-      </c>
-      <c r="M9" t="s">
-        <v>98</v>
       </c>
       <c r="N9" t="s">
         <v>27</v>
@@ -1229,43 +1332,43 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
         <v>99</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10" t="s">
         <v>100</v>
       </c>
-      <c r="C10" t="s">
-        <v>72</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="F10" t="s">
         <v>101</v>
       </c>
-      <c r="E10" t="s">
+      <c r="G10" t="s">
         <v>102</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" t="s">
+        <v>45</v>
+      </c>
+      <c r="I10" t="s">
+        <v>22</v>
+      </c>
+      <c r="J10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" t="s">
         <v>103</v>
       </c>
-      <c r="G10" t="s">
-        <v>76</v>
-      </c>
-      <c r="H10" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" t="s">
-        <v>77</v>
-      </c>
-      <c r="J10" t="s">
-        <v>87</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>104</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>105</v>
-      </c>
-      <c r="M10" t="s">
-        <v>106</v>
       </c>
       <c r="N10" t="s">
         <v>27</v>
@@ -1273,34 +1376,34 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" t="s">
         <v>107</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" t="s">
         <v>108</v>
       </c>
-      <c r="C11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>109</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>110</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
+        <v>102</v>
+      </c>
+      <c r="H11" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" t="s">
         <v>111</v>
       </c>
-      <c r="G11" t="s">
-        <v>76</v>
-      </c>
-      <c r="H11" t="s">
-        <v>35</v>
-      </c>
-      <c r="I11" t="s">
-        <v>36</v>
-      </c>
       <c r="J11" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="K11" t="s">
         <v>112</v>
@@ -1323,19 +1426,19 @@
         <v>116</v>
       </c>
       <c r="C12" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="D12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G12" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="H12" t="s">
         <v>21</v>
@@ -1344,16 +1447,16 @@
         <v>22</v>
       </c>
       <c r="J12" t="s">
-        <v>23</v>
+        <v>121</v>
       </c>
       <c r="K12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="N12" t="s">
         <v>27</v>
@@ -1361,45 +1464,177 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="E13" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F13" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G13" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="H13" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="I13" t="s">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="J13" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="K13" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="L13" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="M13" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="N13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" t="s">
+        <v>136</v>
+      </c>
+      <c r="F14" t="s">
+        <v>137</v>
+      </c>
+      <c r="G14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I14" t="s">
+        <v>46</v>
+      </c>
+      <c r="J14" t="s">
+        <v>84</v>
+      </c>
+      <c r="K14" t="s">
+        <v>138</v>
+      </c>
+      <c r="L14" t="s">
+        <v>139</v>
+      </c>
+      <c r="M14" t="s">
+        <v>140</v>
+      </c>
+      <c r="N14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" t="s">
+        <v>142</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" t="s">
+        <v>143</v>
+      </c>
+      <c r="F15" t="s">
+        <v>144</v>
+      </c>
+      <c r="G15" t="s">
+        <v>102</v>
+      </c>
+      <c r="H15" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15" t="s">
+        <v>111</v>
+      </c>
+      <c r="J15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" t="s">
+        <v>145</v>
+      </c>
+      <c r="L15" t="s">
+        <v>146</v>
+      </c>
+      <c r="M15" t="s">
+        <v>147</v>
+      </c>
+      <c r="N15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>148</v>
+      </c>
+      <c r="B16" t="s">
+        <v>149</v>
+      </c>
+      <c r="C16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" t="s">
+        <v>150</v>
+      </c>
+      <c r="E16" t="s">
+        <v>151</v>
+      </c>
+      <c r="F16" t="s">
+        <v>152</v>
+      </c>
+      <c r="G16" t="s">
+        <v>102</v>
+      </c>
+      <c r="H16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16" t="s">
+        <v>111</v>
+      </c>
+      <c r="J16" t="s">
+        <v>47</v>
+      </c>
+      <c r="K16" t="s">
+        <v>112</v>
+      </c>
+      <c r="L16" t="s">
+        <v>153</v>
+      </c>
+      <c r="M16" t="s">
+        <v>154</v>
+      </c>
+      <c r="N16" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1411,18 +1646,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="37" customWidth="1"/>
+    <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
     <col min="5" max="6" width="60" customWidth="1"/>
     <col min="7" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="13" width="60" customWidth="1"/>
+    <col min="11" max="11" width="44" customWidth="1"/>
+    <col min="12" max="13" width="60" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1537,22 +1773,22 @@
         <v>34</v>
       </c>
       <c r="H3" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="J3" t="s">
         <v>23</v>
       </c>
       <c r="K3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" t="s">
         <v>37</v>
-      </c>
-      <c r="L3" t="s">
-        <v>38</v>
-      </c>
-      <c r="M3" t="s">
-        <v>39</v>
       </c>
       <c r="N3" t="s">
         <v>27</v>
@@ -1560,43 +1796,43 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
         <v>40</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>41</v>
       </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>42</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>43</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>44</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>45</v>
       </c>
-      <c r="H4" t="s">
-        <v>21</v>
-      </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="J4" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="K4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="L4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="M4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="N4" t="s">
         <v>27</v>
@@ -1604,34 +1840,34 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="I5" t="s">
         <v>22</v>
       </c>
       <c r="J5" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="K5" t="s">
         <v>57</v>
@@ -1654,7 +1890,7 @@
         <v>61</v>
       </c>
       <c r="C6" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
         <v>62</v>
@@ -1669,22 +1905,22 @@
         <v>65</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I6" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="J6" t="s">
+        <v>47</v>
+      </c>
+      <c r="K6" t="s">
         <v>66</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>67</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>68</v>
-      </c>
-      <c r="M6" t="s">
-        <v>69</v>
       </c>
       <c r="N6" t="s">
         <v>27</v>
@@ -1692,43 +1928,43 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" t="s">
         <v>70</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
         <v>71</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>72</v>
       </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>74</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" t="s">
         <v>75</v>
       </c>
-      <c r="G7" t="s">
+      <c r="M7" t="s">
         <v>76</v>
-      </c>
-      <c r="H7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" t="s">
-        <v>77</v>
-      </c>
-      <c r="J7" t="s">
-        <v>66</v>
-      </c>
-      <c r="K7" t="s">
-        <v>78</v>
-      </c>
-      <c r="L7" t="s">
-        <v>79</v>
-      </c>
-      <c r="M7" t="s">
-        <v>80</v>
       </c>
       <c r="N7" t="s">
         <v>27</v>
@@ -1736,43 +1972,43 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" t="s">
         <v>81</v>
       </c>
-      <c r="B8" t="s">
+      <c r="F8" t="s">
         <v>82</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
         <v>83</v>
-      </c>
-      <c r="D8" t="s">
-        <v>84</v>
-      </c>
-      <c r="E8" t="s">
-        <v>85</v>
-      </c>
-      <c r="F8" t="s">
-        <v>86</v>
-      </c>
-      <c r="G8" t="s">
-        <v>76</v>
       </c>
       <c r="H8" t="s">
         <v>21</v>
       </c>
       <c r="I8" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="J8" t="s">
+        <v>84</v>
+      </c>
+      <c r="K8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L8" t="s">
+        <v>86</v>
+      </c>
+      <c r="M8" t="s">
         <v>87</v>
-      </c>
-      <c r="K8" t="s">
-        <v>88</v>
-      </c>
-      <c r="L8" t="s">
-        <v>89</v>
-      </c>
-      <c r="M8" t="s">
-        <v>90</v>
       </c>
       <c r="N8" t="s">
         <v>27</v>
@@ -1780,43 +2016,43 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" t="s">
         <v>91</v>
       </c>
-      <c r="B9" t="s">
+      <c r="F9" t="s">
         <v>92</v>
       </c>
-      <c r="C9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="G9" t="s">
         <v>93</v>
       </c>
-      <c r="E9" t="s">
+      <c r="H9" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" t="s">
         <v>94</v>
       </c>
-      <c r="F9" t="s">
+      <c r="L9" t="s">
         <v>95</v>
       </c>
-      <c r="G9" t="s">
-        <v>76</v>
-      </c>
-      <c r="H9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I9" t="s">
-        <v>36</v>
-      </c>
-      <c r="J9" t="s">
-        <v>23</v>
-      </c>
-      <c r="K9" t="s">
+      <c r="M9" t="s">
         <v>96</v>
-      </c>
-      <c r="L9" t="s">
-        <v>97</v>
-      </c>
-      <c r="M9" t="s">
-        <v>98</v>
       </c>
       <c r="N9" t="s">
         <v>27</v>
@@ -1824,43 +2060,43 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
         <v>99</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10" t="s">
         <v>100</v>
       </c>
-      <c r="C10" t="s">
-        <v>72</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="F10" t="s">
         <v>101</v>
       </c>
-      <c r="E10" t="s">
+      <c r="G10" t="s">
         <v>102</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" t="s">
+        <v>45</v>
+      </c>
+      <c r="I10" t="s">
+        <v>22</v>
+      </c>
+      <c r="J10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" t="s">
         <v>103</v>
       </c>
-      <c r="G10" t="s">
-        <v>76</v>
-      </c>
-      <c r="H10" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" t="s">
-        <v>77</v>
-      </c>
-      <c r="J10" t="s">
-        <v>87</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>104</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>105</v>
-      </c>
-      <c r="M10" t="s">
-        <v>106</v>
       </c>
       <c r="N10" t="s">
         <v>27</v>
@@ -1868,34 +2104,34 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" t="s">
         <v>107</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" t="s">
         <v>108</v>
       </c>
-      <c r="C11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>109</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>110</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
+        <v>102</v>
+      </c>
+      <c r="H11" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" t="s">
         <v>111</v>
       </c>
-      <c r="G11" t="s">
-        <v>76</v>
-      </c>
-      <c r="H11" t="s">
-        <v>35</v>
-      </c>
-      <c r="I11" t="s">
-        <v>36</v>
-      </c>
       <c r="J11" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="K11" t="s">
         <v>112</v>
@@ -1918,19 +2154,19 @@
         <v>116</v>
       </c>
       <c r="C12" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="D12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G12" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="H12" t="s">
         <v>21</v>
@@ -1939,16 +2175,16 @@
         <v>22</v>
       </c>
       <c r="J12" t="s">
-        <v>23</v>
+        <v>121</v>
       </c>
       <c r="K12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="N12" t="s">
         <v>27</v>
@@ -1956,45 +2192,177 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="E13" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F13" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G13" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="H13" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="I13" t="s">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="J13" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="K13" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="L13" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="M13" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="N13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" t="s">
+        <v>136</v>
+      </c>
+      <c r="F14" t="s">
+        <v>137</v>
+      </c>
+      <c r="G14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I14" t="s">
+        <v>46</v>
+      </c>
+      <c r="J14" t="s">
+        <v>84</v>
+      </c>
+      <c r="K14" t="s">
+        <v>138</v>
+      </c>
+      <c r="L14" t="s">
+        <v>139</v>
+      </c>
+      <c r="M14" t="s">
+        <v>140</v>
+      </c>
+      <c r="N14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" t="s">
+        <v>142</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" t="s">
+        <v>143</v>
+      </c>
+      <c r="F15" t="s">
+        <v>144</v>
+      </c>
+      <c r="G15" t="s">
+        <v>102</v>
+      </c>
+      <c r="H15" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15" t="s">
+        <v>111</v>
+      </c>
+      <c r="J15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" t="s">
+        <v>145</v>
+      </c>
+      <c r="L15" t="s">
+        <v>146</v>
+      </c>
+      <c r="M15" t="s">
+        <v>147</v>
+      </c>
+      <c r="N15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>148</v>
+      </c>
+      <c r="B16" t="s">
+        <v>149</v>
+      </c>
+      <c r="C16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" t="s">
+        <v>150</v>
+      </c>
+      <c r="E16" t="s">
+        <v>151</v>
+      </c>
+      <c r="F16" t="s">
+        <v>152</v>
+      </c>
+      <c r="G16" t="s">
+        <v>102</v>
+      </c>
+      <c r="H16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16" t="s">
+        <v>111</v>
+      </c>
+      <c r="J16" t="s">
+        <v>47</v>
+      </c>
+      <c r="K16" t="s">
+        <v>112</v>
+      </c>
+      <c r="L16" t="s">
+        <v>153</v>
+      </c>
+      <c r="M16" t="s">
+        <v>154</v>
+      </c>
+      <c r="N16" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2006,16 +2374,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="4" max="4" width="49" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2024,7 +2394,49 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>131</v>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -2047,7 +2459,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2055,7 +2467,7 @@
         <v>16</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2063,53 +2475,53 @@
         <v>30</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>167</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="B10">
         <v>6</v>
@@ -2117,23 +2529,23 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="B11">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>135</v>
+        <v>169</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -2142,18 +2554,18 @@
     <row r="14" spans="1:2" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>136</v>
+        <v>170</v>
       </c>
       <c r="B15">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>137</v>
+        <v>171</v>
       </c>
       <c r="B16">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>